<commit_message>
七星172换仓: 卖出能源化工ETF建信 → 买入南方原油LOF(sh501018)@1.9790 (2026-09-24 13:04)
</commit_message>
<xml_diff>
--- a/backtest/results_172/七星172_交易记录_2026.xlsx
+++ b/backtest/results_172/七星172_交易记录_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H256"/>
+  <dimension ref="A1:H260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9126,6 +9126,142 @@
       </c>
       <c r="H256" t="inlineStr"/>
     </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-09-10 11:03</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>卖出</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>豆粕ETF华夏</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>sz159985</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="F257" t="n">
+        <v>2.8126</v>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>盈利保护卖出(回撤超5%)</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-09-10 13:05</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>能源化工ETF建信</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>sz159981</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>1.787</v>
+      </c>
+      <c r="F258" t="n">
+        <v>5.3213</v>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>动量排名第1/38</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:05</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>卖出</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>能源化工ETF建信</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>sz159981</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>1.725</v>
+      </c>
+      <c r="F259" t="n">
+        <v>1.0293</v>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>排名从2→新第1不等,调出</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-09-24 13:05</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>南方原油LOF</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>sh501018</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>1.979</v>
+      </c>
+      <c r="F260" t="n">
+        <v>1.1193</v>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>动量排名第1/38</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
七星172: 2026-10-20 13:05换仓 卖出纳指ETF国泰(sh513100)@2.348(溢价>20%被过滤) 买入标普消费ETF景顺(sz159529)@1.413(动量第1/38)
</commit_message>
<xml_diff>
--- a/backtest/results_172/七星172_交易记录_2026.xlsx
+++ b/backtest/results_172/七星172_交易记录_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H260"/>
+  <dimension ref="A1:H266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9262,6 +9262,210 @@
       </c>
       <c r="H260" t="inlineStr"/>
     </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-09-30 13:05</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>卖出</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>南方原油LOF</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>sh501018</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>1.957</v>
+      </c>
+      <c r="F261" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>排名从3→新第1不等,调出</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-09-30 13:05</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>能源化工ETF建信</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>sz159981</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>1.779</v>
+      </c>
+      <c r="F262" t="n">
+        <v>0.8336</v>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>动量排名第1/38</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-10-15 11:02</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>卖出</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>能源化工ETF建信</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>sz159981</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>1.839</v>
+      </c>
+      <c r="F263" t="n">
+        <v>1.2437</v>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>盈利保护卖出(回撤超5%)</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:05</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>纳指ETF国泰</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>sh513100</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>2.346</v>
+      </c>
+      <c r="F264" t="n">
+        <v>1.4122</v>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>动量排名第1/38</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-10-20 13:05</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>卖出</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>纳指ETF国泰</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>sh513100</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>2.348</v>
+      </c>
+      <c r="F265" t="n">
+        <v>0.7395</v>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>被过滤规则拦截调出: 溢价&gt;20%</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-10-20 13:05</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>标普消费ETF景顺</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>sz159529</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>1.413</v>
+      </c>
+      <c r="F266" t="n">
+        <v>1.3843</v>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>动量排名第1/38</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
七星172: 2026-10-26 13:04换仓 卖出标普消费ETF景顺(1.375) -> 买入南方原油LOF(2.273)
</commit_message>
<xml_diff>
--- a/backtest/results_172/七星172_交易记录_2026.xlsx
+++ b/backtest/results_172/七星172_交易记录_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H266"/>
+  <dimension ref="A1:H268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9466,6 +9466,74 @@
       </c>
       <c r="H266" t="inlineStr"/>
     </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-26 13:05</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>卖出</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>标普消费ETF景顺</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>sz159529</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>1.375</v>
+      </c>
+      <c r="F267" t="n">
+        <v>1.9744</v>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>排名从2→新第1不等,调出</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-26 13:05</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>买入</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>南方原油LOF</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>sh501018</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>2.273</v>
+      </c>
+      <c r="F268" t="n">
+        <v>2.3268</v>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>动量排名第1/38</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>